<commit_message>
saving Electricity in dashboard
</commit_message>
<xml_diff>
--- a/Outputs/PtX_demand_AT.xlsx
+++ b/Outputs/PtX_demand_AT.xlsx
@@ -503,11 +503,19 @@
       <c r="E2" t="n">
         <v>0.002662064146729648</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>0.01066673417812259</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0100849458616752</v>
+      </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>0.003179812794298</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.00382119238217</v>
+      </c>
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -730,16 +738,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Biomass [Solid]</t>
+          <t>Fossil Residuals</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2030</v>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>0.04748099508246478</v>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>0.01236568429895008</v>
+        <v>0.01745129146664355</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -751,18 +761,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fossil Rest</t>
+          <t>Biomass [Solid]</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>2030</v>
       </c>
-      <c r="C13" t="n">
-        <v>0.04748099508246478</v>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>0.01745129146664355</v>
+        <v>0.01236568429895008</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -811,19 +819,19 @@
         <v>0.03441807229750589</v>
       </c>
       <c r="F15" t="n">
-        <v>0.09969632597160048</v>
+        <v>0.1103630601497231</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0020030733012077</v>
+        <v>0.0120880191628829</v>
       </c>
       <c r="H15" t="n">
         <v>0.02979732750124525</v>
       </c>
       <c r="I15" t="n">
-        <v>0.05669717083959917</v>
+        <v>0.05987698363389717</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0029740057738661</v>
+        <v>0.0067951981560361</v>
       </c>
       <c r="K15" t="n">
         <v>0.0011605685644923</v>
@@ -847,11 +855,19 @@
       <c r="E16" t="n">
         <v>0.002863350770741068</v>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>0.0303462664141143</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0118356141697125</v>
+      </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>0.0123101007029516</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.0037685836858441</v>
+      </c>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1078,16 +1094,20 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Biomass [Solid]</t>
+          <t>Fossil Residuals</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>2040</v>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>0.03327587745866158</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7.673861546209083e-20</v>
+      </c>
       <c r="E26" t="n">
-        <v>0.01390636056580271</v>
+        <v>0.01166729413882539</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1099,20 +1119,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Fossil Rest</t>
+          <t>Biomass [Solid]</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2040</v>
       </c>
-      <c r="C27" t="n">
-        <v>0.03327587745866158</v>
-      </c>
-      <c r="D27" t="n">
-        <v>7.673861546209083e-20</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>0.01166729413882539</v>
+        <v>0.01390636056580271</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1161,19 +1177,19 @@
         <v>0.03621520156791942</v>
       </c>
       <c r="F29" t="n">
-        <v>0.03232039497452344</v>
+        <v>0.06266666138863775</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0022916677209212</v>
+        <v>0.0141272818906337</v>
       </c>
       <c r="H29" t="n">
         <v>0.0289101249010305</v>
       </c>
       <c r="I29" t="n">
-        <v>0.02839560971294071</v>
+        <v>0.04070571041589231</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0027772287071803</v>
+        <v>0.0065458123930244</v>
       </c>
       <c r="K29" t="n">
         <v>0.0010853567358991</v>
@@ -1197,11 +1213,19 @@
       <c r="E30" t="n">
         <v>0.003057232938574005</v>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="F30" t="n">
+        <v>0.0353988844847138</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.0132913255392536</v>
+      </c>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>0.0193104046635765</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.0038489451931328</v>
+      </c>
       <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1440,17 +1464,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Biomass [Solid]</t>
+          <t>Fossil Residuals</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>2050</v>
       </c>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="n">
-        <v>0.01548483145203032</v>
-      </c>
+      <c r="D40" t="n">
+        <v>6.906475391588176e-19</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
@@ -1461,17 +1485,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Fossil Rest</t>
+          <t>Biomass [Solid]</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>2050</v>
       </c>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="n">
-        <v>6.906475391588176e-19</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>0.01548483145203032</v>
+      </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
@@ -1516,22 +1540,22 @@
         <v>0.03586413416225002</v>
       </c>
       <c r="E43" t="n">
-        <v>0.03794028478384233</v>
+        <v>0.03794028478384234</v>
       </c>
       <c r="F43" t="n">
-        <v>0.006117491750374807</v>
+        <v>0.04151637623508861</v>
       </c>
       <c r="G43" t="n">
-        <v>0.00242624326801659</v>
+        <v>0.01571756880727019</v>
       </c>
       <c r="H43" t="n">
         <v>0.02764259946079578</v>
       </c>
       <c r="I43" t="n">
-        <v>0.00584199300638264</v>
+        <v>0.02515239766995914</v>
       </c>
       <c r="J43" t="n">
-        <v>0.002608419127480644</v>
+        <v>0.006457364320613444</v>
       </c>
       <c r="K43" t="n">
         <v>0.0009913087869338215</v>

</xml_diff>